<commit_message>
updated archive, school and academic_record table
</commit_message>
<xml_diff>
--- a/SUHR-System/logs/login_logout_log.xlsx
+++ b/SUHR-System/logs/login_logout_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,40 +513,6 @@
         </is>
       </c>
       <c r="C6" t="inlineStr">
-        <is>
-          <t>Login</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2024-11-15 00:10:13</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>111</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Login</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2024-11-15 11:47:01</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>111</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
         <is>
           <t>Login</t>
         </is>

</xml_diff>